<commit_message>
Popravila sem, da dejansko upošteva koordinate, ki jih zahtevaš.
</commit_message>
<xml_diff>
--- a/Rezultati_Optimizacije_250kW.xlsx
+++ b/Rezultati_Optimizacije_250kW.xlsx
@@ -451,12 +451,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>142.690,15 €</t>
+          <t>143.602,43 €</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>26.566,63 €</t>
+          <t>25.654,35 €</t>
         </is>
       </c>
     </row>
@@ -468,17 +468,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>66.267,02 €</t>
+          <t>67.008,18 €</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>55.906,84 €</t>
+          <t>56.799,05 €</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>10.360,18 €</t>
+          <t>10.209,13 €</t>
         </is>
       </c>
     </row>
@@ -495,12 +495,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>19.181,86 €</t>
+          <t>19.235,56 €</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>3.683,37 €</t>
+          <t>3.629,67 €</t>
         </is>
       </c>
     </row>
@@ -517,12 +517,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>720,78 €</t>
+          <t>722,80 €</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>139,10 €</t>
+          <t>137,08 €</t>
         </is>
       </c>
     </row>
@@ -539,12 +539,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>-957,39 €</t>
+          <t>-1.212,81 €</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>957,39 €</t>
+          <t>1.212,81 €</t>
         </is>
       </c>
     </row>
@@ -578,17 +578,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>259.248,90 €</t>
+          <t>259.990,07 €</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>230.070,41 €</t>
+          <t>231.695,48 €</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>29.178,49 €</t>
+          <t>28.294,59 €</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Za konec sem ustvarila še poročilo o uporabi UI.
</commit_message>
<xml_diff>
--- a/Rezultati_Optimizacije_250kW.xlsx
+++ b/Rezultati_Optimizacije_250kW.xlsx
@@ -451,12 +451,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>143.602,43 €</t>
+          <t>142.690,15 €</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>25.654,35 €</t>
+          <t>26.566,63 €</t>
         </is>
       </c>
     </row>
@@ -468,17 +468,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>67.008,18 €</t>
+          <t>66.267,02 €</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>56.799,05 €</t>
+          <t>55.906,84 €</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>10.209,13 €</t>
+          <t>10.360,18 €</t>
         </is>
       </c>
     </row>
@@ -495,12 +495,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>19.235,56 €</t>
+          <t>19.181,86 €</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>3.629,67 €</t>
+          <t>3.683,37 €</t>
         </is>
       </c>
     </row>
@@ -517,12 +517,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>722,80 €</t>
+          <t>720,78 €</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>137,08 €</t>
+          <t>139,10 €</t>
         </is>
       </c>
     </row>
@@ -539,12 +539,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>-1.212,81 €</t>
+          <t>-957,39 €</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>1.212,81 €</t>
+          <t>957,39 €</t>
         </is>
       </c>
     </row>
@@ -578,17 +578,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>259.990,07 €</t>
+          <t>259.248,90 €</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>231.695,48 €</t>
+          <t>230.070,41 €</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>28.294,59 €</t>
+          <t>29.178,49 €</t>
         </is>
       </c>
     </row>

</xml_diff>